<commit_message>
Data pipeline update and updated intermediate/processed data files
Omitting the large combined data files because of size until I set up git LFS or something
</commit_message>
<xml_diff>
--- a/data/2025/metadata/data_inventory.xlsx
+++ b/data/2025/metadata/data_inventory.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/drotto/src/jiflr/data/2025/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51CA62E4-31B3-5041-BE11-E6BE23A784EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FD8D2B0-5900-3441-A75E-30CD4322D807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17820" yWindow="-28300" windowWidth="25060" windowHeight="28300" xr2:uid="{834A5152-98D4-1D4E-9988-BEC817907187}"/>
+    <workbookView xWindow="10940" yWindow="1580" windowWidth="25060" windowHeight="21100" xr2:uid="{834A5152-98D4-1D4E-9988-BEC817907187}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -107,21 +108,6 @@
     <t>F06</t>
   </si>
   <si>
-    <t>Windward-2</t>
-  </si>
-  <si>
-    <t>Windward-1</t>
-  </si>
-  <si>
-    <t>Divide</t>
-  </si>
-  <si>
-    <t>Lee-1</t>
-  </si>
-  <si>
-    <t>Lee-2</t>
-  </si>
-  <si>
     <t>retrieval notes</t>
   </si>
   <si>
@@ -155,21 +141,9 @@
     <t>missing shielded pendant data</t>
   </si>
   <si>
-    <t>1m SN</t>
-  </si>
-  <si>
-    <t>2m SN</t>
-  </si>
-  <si>
     <t>deployment_datetime</t>
   </si>
   <si>
-    <t>0m SN</t>
-  </si>
-  <si>
-    <t>2m unshaded</t>
-  </si>
-  <si>
     <t>Height for unshaded was not 2m. Maybe 0.5m? On Gulliana's wx station</t>
   </si>
   <si>
@@ -246,6 +220,33 @@
   </si>
   <si>
     <t>2m sensor failed after only a few data points</t>
+  </si>
+  <si>
+    <t>windward2</t>
+  </si>
+  <si>
+    <t>windward1</t>
+  </si>
+  <si>
+    <t>divide</t>
+  </si>
+  <si>
+    <t>lee1</t>
+  </si>
+  <si>
+    <t>lee2</t>
+  </si>
+  <si>
+    <t>2m</t>
+  </si>
+  <si>
+    <t>1m</t>
+  </si>
+  <si>
+    <t>2m_unshielded</t>
+  </si>
+  <si>
+    <t>0m_unshielded</t>
   </si>
 </sst>
 </file>
@@ -333,7 +334,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -365,198 +366,12 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="12">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="27" formatCode="m/d/yy\ hh:mm"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -672,6 +487,183 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="27" formatCode="m/d/yy\ hh:mm"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
       <border outline="0">
         <right style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -720,16 +712,16 @@
   <autoFilter ref="A1:K47" xr:uid="{30214729-FAD1-AB4C-91D6-A2D7E03E2CE5}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{D1314852-2294-C84C-828A-C37A76432716}" name="site_type"/>
-    <tableColumn id="2" xr3:uid="{57B08370-AE15-194A-9E89-74600FFA2010}" name="site_id" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{956B5A7B-9B49-6346-8FCA-C17178CA2BCE}" name="2m unshaded" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{7504CBC9-3359-0648-9D3B-0FB0A1252A94}" name="2m SN" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{CB898744-7014-BB43-BAC1-0B15028E3BA2}" name="1m SN" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{150A9C0A-48E9-3C44-9B57-D88CC22BFD34}" name="0m SN" dataDxfId="0"/>
-    <tableColumn id="7" xr3:uid="{BF7B2BE9-C3D1-8142-A770-41D36B9FF6B2}" name="deployment_datetime" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{A1810F1F-E447-B14E-A6CE-B9996DB950E5}" name="retrieval notes" dataDxfId="9"/>
-    <tableColumn id="9" xr3:uid="{E2307612-7D26-CF4E-A08E-3595C0515637}" name="site photos" dataDxfId="8"/>
-    <tableColumn id="10" xr3:uid="{6EDEA866-AA93-4941-8E8D-DF881109FB3E}" name="data" dataDxfId="7"/>
-    <tableColumn id="11" xr3:uid="{B40B1566-540C-5A43-903E-FD3EC9C1F710}" name="notes" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{57B08370-AE15-194A-9E89-74600FFA2010}" name="site_id" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{956B5A7B-9B49-6346-8FCA-C17178CA2BCE}" name="2m_unshielded" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{7504CBC9-3359-0648-9D3B-0FB0A1252A94}" name="2m" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{CB898744-7014-BB43-BAC1-0B15028E3BA2}" name="1m" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{150A9C0A-48E9-3C44-9B57-D88CC22BFD34}" name="0m_unshielded" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{BF7B2BE9-C3D1-8142-A770-41D36B9FF6B2}" name="deployment_datetime" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{A1810F1F-E447-B14E-A6CE-B9996DB950E5}" name="retrieval notes" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{E2307612-7D26-CF4E-A08E-3595C0515637}" name="site photos" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{6EDEA866-AA93-4941-8E8D-DF881109FB3E}" name="data" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{B40B1566-540C-5A43-903E-FD3EC9C1F710}" name="notes" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1055,9 +1047,8 @@
   <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="13.6640625" style="17" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" style="17" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" style="17"/>
+    <col min="2" max="2" width="13.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" customWidth="1"/>
     <col min="7" max="7" width="21.1640625" customWidth="1"/>
     <col min="8" max="8" width="15" style="1" customWidth="1"/>
     <col min="9" max="9" width="12.33203125" customWidth="1"/>
@@ -1066,48 +1057,48 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>40</v>
+        <v>66</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="19" t="s">
-        <v>47</v>
+      <c r="C2" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D2" s="8">
         <v>22133679</v>
@@ -1115,31 +1106,31 @@
       <c r="E2" s="5">
         <v>22133645</v>
       </c>
-      <c r="F2" s="19" t="s">
-        <v>47</v>
+      <c r="F2" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G2" s="6">
         <v>45828.65625</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I2" s="5"/>
-      <c r="J2" s="19" t="s">
-        <v>31</v>
+      <c r="J2" s="8" t="s">
+        <v>26</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="19">
+      <c r="C3" s="8">
         <v>22038780</v>
       </c>
       <c r="D3" s="8">
@@ -1148,32 +1139,32 @@
       <c r="E3" s="8">
         <v>22133682</v>
       </c>
-      <c r="F3" s="19" t="s">
-        <v>47</v>
+      <c r="F3" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G3" s="9">
         <v>45819.701388888891</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I3" s="8"/>
-      <c r="J3" s="19" t="s">
-        <v>31</v>
+      <c r="J3" s="8" t="s">
+        <v>26</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="19" t="s">
-        <v>47</v>
+      <c r="C4" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D4" s="5">
         <v>22133661</v>
@@ -1181,30 +1172,30 @@
       <c r="E4" s="5">
         <v>22133634</v>
       </c>
-      <c r="F4" s="19" t="s">
-        <v>47</v>
+      <c r="F4" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G4" s="6">
         <v>45829.770833333336</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I4" s="5"/>
-      <c r="J4" s="19" t="s">
-        <v>31</v>
+      <c r="J4" s="8" t="s">
+        <v>26</v>
       </c>
       <c r="K4" s="5"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="19" t="s">
-        <v>47</v>
+      <c r="C5" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D5" s="8">
         <v>22133638</v>
@@ -1212,30 +1203,30 @@
       <c r="E5" s="8">
         <v>22133641</v>
       </c>
-      <c r="F5" s="19" t="s">
-        <v>47</v>
+      <c r="F5" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G5" s="9">
         <v>45829.75</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I5" s="8"/>
-      <c r="J5" s="19" t="s">
-        <v>31</v>
+      <c r="J5" s="8" t="s">
+        <v>26</v>
       </c>
       <c r="K5" s="8"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B6" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="19" t="s">
-        <v>47</v>
+      <c r="C6" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D6" s="5">
         <v>22133644</v>
@@ -1243,7 +1234,7 @@
       <c r="E6" s="8">
         <v>22133664</v>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="8">
         <v>10383220</v>
       </c>
       <c r="G6" s="6">
@@ -1252,19 +1243,19 @@
       <c r="H6" s="11"/>
       <c r="I6" s="5"/>
       <c r="J6" s="12" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="K6" s="8"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="19" t="s">
-        <v>47</v>
+      <c r="C7" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D7" s="8">
         <v>22133672</v>
@@ -1272,7 +1263,7 @@
       <c r="E7" s="8">
         <v>22133660</v>
       </c>
-      <c r="F7" s="19">
+      <c r="F7" s="8">
         <v>10568651</v>
       </c>
       <c r="G7" s="9">
@@ -1280,20 +1271,20 @@
       </c>
       <c r="H7" s="11"/>
       <c r="I7" s="8"/>
-      <c r="J7" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K7" s="19"/>
+      <c r="J7" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K7" s="8"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>49</v>
-      </c>
-      <c r="B8" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="19" t="s">
-        <v>47</v>
+      <c r="C8" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D8" s="5">
         <v>22133667</v>
@@ -1301,30 +1292,30 @@
       <c r="E8" s="5">
         <v>22133640</v>
       </c>
-      <c r="F8" s="19">
+      <c r="F8" s="8">
         <v>10568642</v>
       </c>
       <c r="G8" s="6">
         <v>45825.805555555555</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I8" s="5"/>
-      <c r="J8" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K8" s="19"/>
+      <c r="J8" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K8" s="8"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="19" t="s">
-        <v>47</v>
+      <c r="C9" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D9" s="8">
         <v>22133642</v>
@@ -1332,30 +1323,30 @@
       <c r="E9" s="8">
         <v>22133665</v>
       </c>
-      <c r="F9" s="19" t="s">
-        <v>47</v>
+      <c r="F9" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G9" s="9">
         <v>45825.815972222219</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I9" s="8"/>
-      <c r="J9" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K9" s="19"/>
+      <c r="J9" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K9" s="8"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>49</v>
-      </c>
-      <c r="B10" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="19" t="s">
-        <v>47</v>
+      <c r="C10" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D10" s="5">
         <v>22133683</v>
@@ -1363,7 +1354,7 @@
       <c r="E10" s="5">
         <v>22133656</v>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="8">
         <v>9668113</v>
       </c>
       <c r="G10" s="6">
@@ -1371,20 +1362,20 @@
       </c>
       <c r="H10" s="11"/>
       <c r="I10" s="5"/>
-      <c r="J10" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K10" s="19"/>
+      <c r="J10" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K10" s="8"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="19" t="s">
-        <v>47</v>
+      <c r="C11" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D11" s="8">
         <v>22133687</v>
@@ -1392,30 +1383,30 @@
       <c r="E11" s="8">
         <v>22133671</v>
       </c>
-      <c r="F11" s="19" t="s">
-        <v>47</v>
+      <c r="F11" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G11" s="9">
         <v>45828.597222222219</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I11" s="8"/>
-      <c r="J11" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K11" s="19"/>
+      <c r="J11" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K11" s="8"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>49</v>
-      </c>
-      <c r="B12" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="19" t="s">
-        <v>47</v>
+      <c r="C12" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D12" s="5">
         <v>22133680</v>
@@ -1423,32 +1414,32 @@
       <c r="E12" s="5">
         <v>22133663</v>
       </c>
-      <c r="F12" s="19" t="s">
-        <v>47</v>
+      <c r="F12" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G12" s="6">
         <v>45820.713194444441</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="I12" s="5"/>
-      <c r="J12" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K12" s="19" t="s">
-        <v>51</v>
+      <c r="J12" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="19" t="s">
-        <v>47</v>
+      <c r="C13" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D13" s="8">
         <v>22133635</v>
@@ -1456,30 +1447,30 @@
       <c r="E13" s="8">
         <v>22133624</v>
       </c>
-      <c r="F13" s="19" t="s">
-        <v>47</v>
+      <c r="F13" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G13" s="9">
         <v>45820.697916666664</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I13" s="8"/>
-      <c r="J13" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K13" s="19"/>
+      <c r="J13" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K13" s="8"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="19" t="s">
-        <v>47</v>
+      <c r="C14" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D14" s="5">
         <v>22133637</v>
@@ -1487,30 +1478,30 @@
       <c r="E14" s="5">
         <v>22133625</v>
       </c>
-      <c r="F14" s="19" t="s">
-        <v>47</v>
+      <c r="F14" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G14" s="6">
         <v>45828.715277777781</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I14" s="5"/>
-      <c r="J14" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K14" s="19"/>
+      <c r="J14" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K14" s="8"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>49</v>
-      </c>
-      <c r="B15" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="19" t="s">
-        <v>47</v>
+      <c r="C15" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D15" s="8">
         <v>22133646</v>
@@ -1518,30 +1509,30 @@
       <c r="E15" s="8">
         <v>22133652</v>
       </c>
-      <c r="F15" s="19" t="s">
-        <v>47</v>
+      <c r="F15" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G15" s="9">
         <v>45829.722222222219</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I15" s="8"/>
-      <c r="J15" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K15" s="19"/>
+      <c r="J15" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K15" s="8"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B16" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="19" t="s">
-        <v>47</v>
+      <c r="C16" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D16" s="5">
         <v>22133659</v>
@@ -1549,30 +1540,30 @@
       <c r="E16" s="5">
         <v>22133686</v>
       </c>
-      <c r="F16" s="19" t="s">
-        <v>47</v>
+      <c r="F16" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G16" s="6">
         <v>45829.559027777781</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I16" s="5"/>
-      <c r="J16" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K16" s="19"/>
+      <c r="J16" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K16" s="8"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>49</v>
-      </c>
-      <c r="B17" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="19" t="s">
-        <v>47</v>
+      <c r="C17" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D17" s="8">
         <v>22133630</v>
@@ -1580,30 +1571,30 @@
       <c r="E17" s="8">
         <v>22133636</v>
       </c>
-      <c r="F17" s="19" t="s">
-        <v>47</v>
+      <c r="F17" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G17" s="9">
         <v>45829.517361111109</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I17" s="8"/>
-      <c r="J17" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K17" s="19"/>
+      <c r="J17" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K17" s="8"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>49</v>
-      </c>
-      <c r="B18" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="19" t="s">
-        <v>47</v>
+      <c r="C18" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D18" s="5">
         <v>22133653</v>
@@ -1611,30 +1602,30 @@
       <c r="E18" s="5">
         <v>22133647</v>
       </c>
-      <c r="F18" s="19" t="s">
-        <v>47</v>
+      <c r="F18" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G18" s="6">
         <v>45829.690972222219</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="I18" s="5"/>
-      <c r="J18" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K18" s="19"/>
+      <c r="J18" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K18" s="8"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B19" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="19" t="s">
-        <v>47</v>
+      <c r="C19" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D19" s="8">
         <v>22133674</v>
@@ -1642,30 +1633,30 @@
       <c r="E19" s="8">
         <v>22133626</v>
       </c>
-      <c r="F19" s="19" t="s">
-        <v>47</v>
+      <c r="F19" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G19" s="9">
         <v>45829.642361111109</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="I19" s="8"/>
-      <c r="J19" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K19" s="19"/>
+      <c r="J19" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K19" s="8"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>49</v>
-      </c>
-      <c r="B20" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="19" t="s">
-        <v>47</v>
+      <c r="C20" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D20" s="5">
         <v>22133643</v>
@@ -1673,30 +1664,30 @@
       <c r="E20" s="5">
         <v>22133657</v>
       </c>
-      <c r="F20" s="19" t="s">
-        <v>47</v>
+      <c r="F20" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G20" s="6">
         <v>45829.614583333336</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K20" s="19"/>
+        <v>26</v>
+      </c>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K20" s="8"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>49</v>
-      </c>
-      <c r="B21" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="19" t="s">
-        <v>47</v>
+      <c r="C21" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D21" s="8">
         <v>22133685</v>
@@ -1704,30 +1695,30 @@
       <c r="E21" s="8">
         <v>22133668</v>
       </c>
-      <c r="F21" s="19" t="s">
-        <v>47</v>
+      <c r="F21" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G21" s="9">
         <v>45830.489583333336</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I21" s="19"/>
-      <c r="J21" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K21" s="19"/>
+        <v>26</v>
+      </c>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K21" s="8"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>49</v>
-      </c>
-      <c r="B22" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="19" t="s">
-        <v>47</v>
+      <c r="C22" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D22" s="5">
         <v>22133669</v>
@@ -1735,30 +1726,30 @@
       <c r="E22" s="5">
         <v>22133629</v>
       </c>
-      <c r="F22" s="19" t="s">
-        <v>47</v>
+      <c r="F22" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G22" s="6">
         <v>45830.513888888891</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="I22" s="19"/>
-      <c r="J22" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K22" s="19"/>
+        <v>26</v>
+      </c>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K22" s="8"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>49</v>
-      </c>
-      <c r="B23" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C23" s="19" t="s">
-        <v>47</v>
+      <c r="C23" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D23" s="8">
         <v>22133673</v>
@@ -1766,30 +1757,30 @@
       <c r="E23" s="8">
         <v>22133676</v>
       </c>
-      <c r="F23" s="19">
+      <c r="F23" s="8">
         <v>10908287</v>
       </c>
       <c r="G23" s="9">
         <v>45830.625</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K23" s="19"/>
+        <v>26</v>
+      </c>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K23" s="8"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>49</v>
-      </c>
-      <c r="B24" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="C24" s="19" t="s">
-        <v>47</v>
+        <v>40</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D24" s="5">
         <v>22133648</v>
@@ -1797,30 +1788,30 @@
       <c r="E24" s="5">
         <v>22133675</v>
       </c>
-      <c r="F24" s="19" t="s">
-        <v>47</v>
+      <c r="F24" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G24" s="6">
         <v>45830.770833333336</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="I24" s="19"/>
-      <c r="J24" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K24" s="19"/>
+        <v>26</v>
+      </c>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K24" s="8"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>49</v>
-      </c>
-      <c r="B25" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>47</v>
+        <v>40</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="D25" s="8">
         <v>22133628</v>
@@ -1828,449 +1819,423 @@
       <c r="E25" s="8">
         <v>22133666</v>
       </c>
-      <c r="F25" s="19" t="s">
-        <v>47</v>
+      <c r="F25" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="G25" s="9">
         <v>45830.784722222219</v>
       </c>
-      <c r="H25" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I25" s="19"/>
-      <c r="J25" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K25" s="19"/>
+      <c r="H25" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K25" s="8"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>49</v>
-      </c>
-      <c r="B26" s="18" t="s">
-        <v>52</v>
-      </c>
-      <c r="C26" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="D26" s="19">
+        <v>40</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" s="8">
         <v>22133651</v>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="8">
         <v>10568620</v>
       </c>
-      <c r="F26" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="G26" s="20">
+      <c r="F26" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G26" s="9">
         <v>45831.229166666664</v>
       </c>
-      <c r="H26" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I26" s="19"/>
-      <c r="J26" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K26" s="19" t="s">
-        <v>46</v>
+      <c r="H26" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K26" s="8" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>49</v>
-      </c>
-      <c r="B27" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="C27" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="D27" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="E27" s="19">
+        <v>40</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E27" s="8">
         <v>10383462</v>
       </c>
-      <c r="F27" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="G27" s="20">
+      <c r="F27" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G27" s="9">
         <v>45831.229166666664</v>
       </c>
-      <c r="H27" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I27" s="19"/>
-      <c r="J27" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K27" s="19"/>
+      <c r="H27" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K27" s="8"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>49</v>
-      </c>
-      <c r="B28" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="C28" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="D28" s="19">
+        <v>40</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D28" s="8">
         <v>22133670</v>
       </c>
-      <c r="E28" s="19">
+      <c r="E28" s="8">
         <v>22133655</v>
       </c>
-      <c r="F28" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="G28" s="20">
+      <c r="F28" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G28" s="9">
         <v>45831.21875</v>
       </c>
-      <c r="H28" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I28" s="19"/>
-      <c r="J28" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K28" s="19" t="s">
-        <v>45</v>
+      <c r="H28" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K28" s="8" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B29" s="18"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="20"/>
-      <c r="H29" s="21"/>
-      <c r="I29" s="19"/>
-      <c r="J29" s="21"/>
-      <c r="K29" s="19"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="8"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B30" s="18"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="20"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="19"/>
-      <c r="J30" s="21"/>
-      <c r="K30" s="19"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="8"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>50</v>
-      </c>
-      <c r="B31" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C31" s="19">
+        <v>41</v>
+      </c>
+      <c r="B31" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="8">
         <v>22038781</v>
       </c>
-      <c r="D31" s="19">
+      <c r="D31" s="8">
         <v>22133681</v>
       </c>
-      <c r="E31" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="F31" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="G31" s="20">
+      <c r="E31" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G31" s="9">
         <v>45830.739583333336</v>
       </c>
       <c r="H31" s="11"/>
-      <c r="I31" s="19"/>
+      <c r="I31" s="8"/>
       <c r="J31" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="K31" s="19"/>
+        <v>33</v>
+      </c>
+      <c r="K31" s="8"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>50</v>
-      </c>
-      <c r="B32" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="C32" s="19">
+        <v>41</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C32" s="8">
         <v>22038779</v>
       </c>
-      <c r="D32" s="19">
+      <c r="D32" s="8">
         <v>22133658</v>
       </c>
-      <c r="E32" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="F32" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="G32" s="20">
+      <c r="E32" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G32" s="9">
         <v>45827.774305555555</v>
       </c>
-      <c r="H32" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I32" s="19"/>
-      <c r="J32" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="K32" s="19"/>
+      <c r="H32" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I32" s="8"/>
+      <c r="J32" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K32" s="8"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>50</v>
-      </c>
-      <c r="B33" s="18" t="s">
-        <v>25</v>
-      </c>
-      <c r="C33" s="19">
+        <v>41</v>
+      </c>
+      <c r="B33" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="C33" s="8">
         <v>22038776</v>
       </c>
-      <c r="D33" s="19">
+      <c r="D33" s="8">
         <v>22133654</v>
       </c>
-      <c r="E33" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="F33" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="G33" s="20">
+      <c r="E33" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G33" s="9">
         <v>45827.6875</v>
       </c>
-      <c r="H33" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I33" s="19"/>
-      <c r="J33" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="K33" s="19"/>
+      <c r="H33" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I33" s="8"/>
+      <c r="J33" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K33" s="8"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>50</v>
-      </c>
-      <c r="B34" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="C34" s="19">
+        <v>41</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C34" s="8">
         <v>22038777</v>
       </c>
-      <c r="D34" s="19">
+      <c r="D34" s="8">
         <v>22133649</v>
       </c>
-      <c r="E34" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="F34" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="G34" s="20">
+      <c r="E34" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G34" s="9">
         <v>45825.791666666664</v>
       </c>
-      <c r="H34" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I34" s="19"/>
-      <c r="J34" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="K34" s="19"/>
+      <c r="H34" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I34" s="8"/>
+      <c r="J34" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K34" s="8"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>50</v>
-      </c>
-      <c r="B35" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="C35" s="19">
+        <v>41</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" s="8">
         <v>22038778</v>
       </c>
-      <c r="D35" s="19">
+      <c r="D35" s="8">
         <v>22133662</v>
       </c>
-      <c r="E35" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="F35" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="G35" s="20">
+      <c r="E35" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G35" s="9">
         <v>45825.590277777781</v>
       </c>
-      <c r="H35" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="I35" s="19"/>
-      <c r="J35" s="21" t="s">
-        <v>31</v>
-      </c>
-      <c r="K35" s="19"/>
+      <c r="H35" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I35" s="8"/>
+      <c r="J35" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K35" s="8"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B36" s="18"/>
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="19"/>
-      <c r="G36" s="20"/>
-      <c r="H36" s="21"/>
-      <c r="I36" s="19"/>
-      <c r="J36" s="21"/>
-      <c r="K36" s="19"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="10"/>
+      <c r="K36" s="8"/>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>55</v>
-      </c>
-      <c r="B37" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="C37" s="19"/>
+        <v>46</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C37" s="8"/>
       <c r="D37" s="12"/>
-      <c r="E37" s="19"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="20"/>
-      <c r="H37" s="21"/>
-      <c r="I37" s="19"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="8"/>
       <c r="J37" s="16"/>
-      <c r="K37" s="19"/>
+      <c r="K37" s="8"/>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>55</v>
-      </c>
-      <c r="B38" s="17" t="s">
-        <v>57</v>
+        <v>46</v>
+      </c>
+      <c r="B38" t="s">
+        <v>48</v>
       </c>
       <c r="D38" s="13"/>
-      <c r="E38" s="17"/>
-      <c r="G38" s="17"/>
-      <c r="H38" s="22"/>
-      <c r="I38" s="17"/>
       <c r="J38" s="15"/>
-      <c r="K38" s="17"/>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>55</v>
-      </c>
-      <c r="B39" s="17" t="s">
-        <v>59</v>
+        <v>46</v>
+      </c>
+      <c r="B39" t="s">
+        <v>50</v>
       </c>
       <c r="D39" s="13"/>
-      <c r="E39" s="17"/>
-      <c r="G39" s="17"/>
-      <c r="H39" s="22"/>
-      <c r="I39" s="17"/>
       <c r="J39" s="15"/>
-      <c r="K39" s="17"/>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>55</v>
-      </c>
-      <c r="B40" s="17" t="s">
-        <v>58</v>
+        <v>46</v>
+      </c>
+      <c r="B40" t="s">
+        <v>49</v>
       </c>
       <c r="D40" s="13"/>
-      <c r="E40" s="17"/>
-      <c r="G40" s="17"/>
-      <c r="H40" s="22"/>
-      <c r="I40" s="17"/>
       <c r="J40" s="15"/>
-      <c r="K40" s="17"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>55</v>
-      </c>
-      <c r="B41" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="C41" s="19"/>
+        <v>46</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="C41" s="8"/>
       <c r="D41" s="14"/>
       <c r="E41" s="8"/>
-      <c r="F41" s="19"/>
+      <c r="F41" s="8"/>
       <c r="G41" s="9"/>
-      <c r="H41" s="21"/>
-      <c r="I41" s="19"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="8"/>
       <c r="J41" s="11"/>
-      <c r="K41" s="19"/>
+      <c r="K41" s="8"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>55</v>
-      </c>
-      <c r="B42" s="17" t="s">
-        <v>61</v>
+        <v>46</v>
+      </c>
+      <c r="B42" t="s">
+        <v>52</v>
       </c>
       <c r="D42" s="13"/>
-      <c r="H42" s="22"/>
       <c r="J42" s="15"/>
-      <c r="K42" s="17"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>55</v>
-      </c>
-      <c r="B43" s="17" t="s">
-        <v>60</v>
+        <v>46</v>
+      </c>
+      <c r="B43" t="s">
+        <v>51</v>
       </c>
       <c r="D43" s="13"/>
-      <c r="H43" s="22"/>
       <c r="J43" s="15"/>
-      <c r="K43" s="17"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>55</v>
-      </c>
-      <c r="B44" s="17" t="s">
-        <v>62</v>
+        <v>46</v>
+      </c>
+      <c r="B44" t="s">
+        <v>53</v>
       </c>
       <c r="D44" s="13"/>
-      <c r="H44" s="22"/>
       <c r="J44" s="15"/>
-      <c r="K44" s="17"/>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="H45" s="22"/>
-      <c r="K45" s="17"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>64</v>
-      </c>
-      <c r="B46" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="H46" s="22"/>
+        <v>55</v>
+      </c>
+      <c r="B46" t="s">
+        <v>57</v>
+      </c>
       <c r="J46" s="15"/>
       <c r="K46" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>64</v>
-      </c>
-      <c r="B47" s="17" t="s">
-        <v>65</v>
+        <v>55</v>
+      </c>
+      <c r="B47" t="s">
+        <v>56</v>
       </c>
       <c r="J47" s="15"/>
       <c r="K47" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated data processing pipeline output
</commit_message>
<xml_diff>
--- a/data/2025/metadata/data_inventory.xlsx
+++ b/data/2025/metadata/data_inventory.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/drotto/src/jiflr/data/2025/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FD8D2B0-5900-3441-A75E-30CD4322D807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53DA5416-EEC2-8943-8E6A-D66EABF17990}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10940" yWindow="1580" windowWidth="25060" windowHeight="21100" xr2:uid="{834A5152-98D4-1D4E-9988-BEC817907187}"/>
+    <workbookView xWindow="1100" yWindow="880" windowWidth="34900" windowHeight="22500" activeTab="1" xr2:uid="{834A5152-98D4-1D4E-9988-BEC817907187}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="98">
   <si>
     <t>site_id</t>
   </si>
@@ -247,6 +248,90 @@
   </si>
   <si>
     <t>0m_unshielded</t>
+  </si>
+  <si>
+    <t>deployment time from photos</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>TKG4 2m</t>
+  </si>
+  <si>
+    <t>Site does not exist on caltopo</t>
+  </si>
+  <si>
+    <t>start time match .hobo file?</t>
+  </si>
+  <si>
+    <t>SN match .hobo file?</t>
+  </si>
+  <si>
+    <t>.hobo file serial number</t>
+  </si>
+  <si>
+    <t>.hobo file sensor name</t>
+  </si>
+  <si>
+    <t>C02 2m</t>
+  </si>
+  <si>
+    <t>.hobo file name</t>
+  </si>
+  <si>
+    <t>conclusion</t>
+  </si>
+  <si>
+    <t>Sensors with this label are mislabelled</t>
+  </si>
+  <si>
+    <t>TKG4 = A02</t>
+  </si>
+  <si>
+    <t>C01 2m</t>
+  </si>
+  <si>
+    <t>C01 (file does not exist)</t>
+  </si>
+  <si>
+    <t>This is correctly identified as G04</t>
+  </si>
+  <si>
+    <t>This is correctly identified as C02</t>
+  </si>
+  <si>
+    <t>This is correctly identified as G03</t>
+  </si>
+  <si>
+    <t>implied serial number from data_inventory sheet</t>
+  </si>
+  <si>
+    <t>A02 2m</t>
+  </si>
+  <si>
+    <t>G03 2m</t>
+  </si>
+  <si>
+    <t>G04 2m</t>
+  </si>
+  <si>
+    <t>G04 1m</t>
+  </si>
+  <si>
+    <t>C01 1m</t>
+  </si>
+  <si>
+    <t>"G03 100" is written on sensor and bag</t>
+  </si>
+  <si>
+    <t>This is correctly identified as G04 1m</t>
+  </si>
+  <si>
+    <t>"G03 200" is written on sensor and bag. Geotagged photo + personal memory agree that this site is at the bottom of the C10 hill</t>
+  </si>
+  <si>
+    <t>"A02 200" written on sensor and bag. By photo geotag, G04 -&gt; G03 order, and jeremy sensors at 1m, this is not the site at the bottom of the C10 hill</t>
   </si>
 </sst>
 </file>
@@ -334,7 +419,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -367,6 +452,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1047,6 +1136,7 @@
   <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.6640625" customWidth="1"/>
     <col min="3" max="3" width="14.1640625" customWidth="1"/>
     <col min="7" max="7" width="21.1640625" customWidth="1"/>
@@ -2245,4 +2335,204 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64892D2D-4B40-DA40-B7E4-D68118DD7E28}">
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.1640625" customWidth="1"/>
+    <col min="2" max="2" width="30.1640625" customWidth="1"/>
+    <col min="3" max="3" width="31.6640625" customWidth="1"/>
+    <col min="4" max="4" width="21" customWidth="1"/>
+    <col min="5" max="5" width="16.1640625" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
+    <col min="8" max="8" width="19.1640625" style="19" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" style="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" s="19" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A1" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="E1" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="G1" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="H1" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="18">
+        <v>45819.666666666664</v>
+      </c>
+      <c r="C2">
+        <v>22133650</v>
+      </c>
+      <c r="D2">
+        <v>22133650</v>
+      </c>
+      <c r="E2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G2" t="s">
+        <v>72</v>
+      </c>
+      <c r="I2" s="19" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>84</v>
+      </c>
+      <c r="H3" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="I3" s="19" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="68" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="18">
+        <v>45828.711111111108</v>
+      </c>
+      <c r="C4">
+        <v>22133637</v>
+      </c>
+      <c r="D4">
+        <v>22133637</v>
+      </c>
+      <c r="E4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" t="s">
+        <v>71</v>
+      </c>
+      <c r="G4" t="s">
+        <v>78</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="136" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" s="18">
+        <v>45831.260416666664</v>
+      </c>
+      <c r="C5">
+        <v>22133651</v>
+      </c>
+      <c r="D5">
+        <v>22133651</v>
+      </c>
+      <c r="E5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" t="s">
+        <v>71</v>
+      </c>
+      <c r="G5" t="s">
+        <v>78</v>
+      </c>
+      <c r="H5" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="119" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="18">
+        <v>45831.220833333333</v>
+      </c>
+      <c r="C6">
+        <v>22133670</v>
+      </c>
+      <c r="D6">
+        <v>22133670</v>
+      </c>
+      <c r="E6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" t="s">
+        <v>83</v>
+      </c>
+      <c r="H6" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="I6" s="19" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="51" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" s="18">
+        <v>45831.220138888886</v>
+      </c>
+      <c r="C7">
+        <v>22133655</v>
+      </c>
+      <c r="D7">
+        <v>22133655</v>
+      </c>
+      <c r="E7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F7" t="s">
+        <v>71</v>
+      </c>
+      <c r="G7" t="s">
+        <v>93</v>
+      </c>
+      <c r="H7" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="I7" s="19" t="s">
+        <v>95</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
 </file>
</xml_diff>